<commit_message>
README completo por pestaña + regression test + capturas actualizadas
- tests/regression_test.py: 21 chequeos sin browser (datos con DV válido
  CPF/CNPJ/RUT/CI, comparador de dealers, schedule semanal, regex, imports).
- README: sección de regression test, chequeo de CTA/links rotos de la TY page
  (columnas "TYP con CTA" y "LINK ISSUE TYP"), diálogo de Configuración avanzada,
  y cta_evidence/ en la estructura de carpetas.
- Capturas: recapturadas contra la UI actual (los tabs habían cambiado de nombre),
  con email y usuario de LambdaTest reemplazados por placeholders.
- .gitignore: excluye Excels reales de ranking de dealers.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/Lead_information_Formulario_Brasil_Chrome.xlsx
+++ b/data/Lead_information_Formulario_Brasil_Chrome.xlsx
@@ -64,34 +64,34 @@
     <t>Dispositivo</t>
   </si>
   <si>
-    <t>https://www.chevrolet.com.br/content/chevrolet/sa/br/pt/testing-folder/raq-eletricos-revamp.html</t>
-  </si>
-  <si>
-    <t>https://secure-developments.com/commonwealth/brasil/gm_forms/raq-eletricos-revamp</t>
-  </si>
-  <si>
-    <t>Rodrigo</t>
-  </si>
-  <si>
-    <t>Nuñez</t>
-  </si>
-  <si>
-    <t>26495567065</t>
-  </si>
-  <si>
-    <t>65983616000175</t>
-  </si>
-  <si>
-    <t>65042120</t>
-  </si>
-  <si>
-    <t>88930676265</t>
-  </si>
-  <si>
-    <t>rodrigonunez_br25_chrome@mrm.com</t>
-  </si>
-  <si>
-    <t>GW2MU1FM0XJA82W46</t>
+    <t>https://www.chevrolet.com.br/solicitar-contato</t>
+  </si>
+  <si>
+    <t>https://secure-developments.com/commonwealth/brasil/gm_forms/raq</t>
+  </si>
+  <si>
+    <t>Ramón</t>
+  </si>
+  <si>
+    <t>Quispe Soto</t>
+  </si>
+  <si>
+    <t>67355913999</t>
+  </si>
+  <si>
+    <t>82766347000104</t>
+  </si>
+  <si>
+    <t>69060118</t>
+  </si>
+  <si>
+    <t>36904207741</t>
+  </si>
+  <si>
+    <t>ramonquispesoto_br51_chrome@mrm.com</t>
+  </si>
+  <si>
+    <t>D0DM0BY48VTGVDG4P</t>
   </si>
   <si>
     <t>chrome</t>

</xml_diff>